<commit_message>
Restructure docs and make construction resolution codeSpace-aware
Docs:
- Add EPLUS_RULES.md as the single EnergyPlus rulebook; remove RULES_code.md
- Add COVERAGE.md (Energy ADE model coverage + gaps)
- Move MAPPING.md and SESSION_HANDOFF.md to repo root; remove process.md
- Refresh CLAUDE.md to current structure

Constructions/materials:
- Resolve by (codeSpace, code) identity, never the bare code
- Excel/DB lookup keyed on codeSpace via a required code_space column in construction_db.xlsx
- Add in-file LayeredConstructionLibrary resolution by (codeSpace, code)
- Drop the silent bare-code fallback so a misconfigured DB fails loudly

Pipeline:
- Two-view middle layer (trace + idf)
- Ignore test_outputs/; add input sample GML files
</commit_message>
<xml_diff>
--- a/citygml2idf/input/construction_db.xlsx
+++ b/citygml2idf/input/construction_db.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,6 +451,11 @@
           <t>material_name</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>code_space</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -651,6 +656,11 @@
           <t>EXCEL_ADE_Wall_L1_Plaster_10mm</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>layered_constr_library_codeSpace</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -671,6 +681,11 @@
           <t>EXCEL_ADE_Wall_L2_Brick_300mm</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>layered_constr_library_codeSpace</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -691,6 +706,11 @@
           <t>EXCEL_ADE_Wall_L3_AirGap_30mm</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>layered_constr_library_codeSpace</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -711,6 +731,11 @@
           <t>EXCEL_ADE_Wall_L4_Insulation_80mm</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>layered_constr_library_codeSpace</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -729,6 +754,11 @@
       <c r="D15" t="inlineStr">
         <is>
           <t>EXCEL_ADE_Wall_L5_Render_20mm</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>layered_constr_library_codeSpace</t>
         </is>
       </c>
     </row>
@@ -816,7 +846,6 @@
           <t>MediumRough</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -846,7 +875,6 @@
           <t>MediumRough</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -876,7 +904,6 @@
           <t>MediumSmooth</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -906,7 +933,6 @@
           <t>MediumRough</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -936,7 +962,6 @@
           <t>MediumSmooth</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -949,11 +974,6 @@
           <t>Material:AirGap</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
         <v>0.15</v>
       </c>
@@ -969,11 +989,6 @@
           <t>Material:AirGap</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>0.18</v>
       </c>
@@ -989,10 +1004,6 @@
           <t>Material:NoMass</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>Rough</t>
@@ -1013,10 +1024,6 @@
           <t>Material:NoMass</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>MediumRough</t>
@@ -1054,7 +1061,6 @@
           <t>MediumRough</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1084,7 +1090,6 @@
           <t>MediumRough</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1097,11 +1102,6 @@
           <t>Material:AirGap</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
         <v>0.15</v>
       </c>
@@ -1134,7 +1134,6 @@
           <t>MediumRough</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1164,7 +1163,6 @@
           <t>MediumRough</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>